<commit_message>
fix(balance): correct ten-commandment boss order and health bases
Patch only the ten-commandment records in both inputs and runtime data. Correct the final four health bases, preserve every formula and unrelated encounter, and validate all ten standard N2 results.
</commit_message>
<xml_diff>
--- a/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
+++ b/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
@@ -1469,17 +1469,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>信仰</t>
+          <t>真实</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25104960</v>
+        <v>19104960</v>
       </c>
       <c r="C8" t="n">
-        <v>550</v>
+        <v>500</v>
       </c>
       <c r="D8" t="n">
-        <v>1200000</v>
+        <v>1000000</v>
       </c>
       <c r="E8" t="n">
         <v>0.5</v>
@@ -1506,17 +1506,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>安息</t>
+          <t>信仰</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>30104960</v>
+        <v>25104960</v>
       </c>
       <c r="C9" t="n">
-        <v>600</v>
+        <v>550</v>
       </c>
       <c r="D9" t="n">
-        <v>1400000</v>
+        <v>1200000</v>
       </c>
       <c r="E9" t="n">
         <v>0.5</v>
@@ -1543,17 +1543,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>忍耐</t>
+          <t>安息</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>35104960</v>
+        <v>30104960</v>
       </c>
       <c r="C10" t="n">
-        <v>650</v>
+        <v>600</v>
       </c>
       <c r="D10" t="n">
-        <v>2000000</v>
+        <v>1400000</v>
       </c>
       <c r="E10" t="n">
         <v>0.5</v>
@@ -1580,17 +1580,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>无欲</t>
+          <t>忍耐</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>40104960</v>
+        <v>35104960</v>
       </c>
       <c r="C11" t="n">
-        <v>700</v>
+        <v>650</v>
       </c>
       <c r="D11" t="n">
-        <v>2200000</v>
+        <v>2000000</v>
       </c>
       <c r="E11" t="n">
         <v>0.5</v>
@@ -1617,17 +1617,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>戒杀</t>
+          <t>无欲</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>45104960</v>
+        <v>40104960</v>
       </c>
       <c r="C12" t="n">
-        <v>750</v>
+        <v>700</v>
       </c>
       <c r="D12" t="n">
-        <v>2400000</v>
+        <v>2200000</v>
       </c>
       <c r="E12" t="n">
         <v>0.5</v>
@@ -1654,17 +1654,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>沉默</t>
+          <t>戒杀</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>50104960</v>
+        <v>45104960</v>
       </c>
       <c r="C13" t="n">
-        <v>800</v>
+        <v>750</v>
       </c>
       <c r="D13" t="n">
-        <v>2600000</v>
+        <v>2400000</v>
       </c>
       <c r="E13" t="n">
         <v>0.5</v>
@@ -1691,17 +1691,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>纯洁</t>
+          <t>沉默</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>55104960</v>
+        <v>50100000</v>
       </c>
       <c r="C14" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="D14" t="n">
-        <v>2800000</v>
+        <v>2600000</v>
       </c>
       <c r="E14" t="n">
         <v>0.5</v>
@@ -1728,17 +1728,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>敬神</t>
+          <t>纯洁</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>60104960</v>
+        <v>55100000</v>
       </c>
       <c r="C15" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="D15" t="n">
-        <v>4000000</v>
+        <v>2800000</v>
       </c>
       <c r="E15" t="n">
         <v>0.5</v>
@@ -1765,17 +1765,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>真实</t>
+          <t>敬神</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>19104960</v>
+        <v>60100000</v>
       </c>
       <c r="C16" t="n">
-        <v>500</v>
+        <v>1200</v>
       </c>
       <c r="D16" t="n">
-        <v>1000000</v>
+        <v>4000000</v>
       </c>
       <c r="E16" t="n">
         <v>0.5</v>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>70104960</v>
+        <v>70100000</v>
       </c>
       <c r="C17" t="n">
         <v>1400</v>

</xml_diff>

<commit_message>
Correct rich N10 wave eight flying monster health to 1.42 million
</commit_message>
<xml_diff>
--- a/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
+++ b/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
@@ -1,29 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模式与难度" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数量与间隔" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="出怪类型" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="波次小怪基础值" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="进攻BOSS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="挑战建筑" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="天灾首怪与精英" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="特殊轮换怪" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="四房" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="转生BOSS" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="特殊BOSS" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="存档挑战" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="虚空之影" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="修正表" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="解锁条件" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="示例" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="模式与难度" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="数量与间隔" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="出怪类型" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="波次小怪基础值" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="进攻BOSS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="挑战建筑" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="天灾首怪与精英" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="特殊轮换怪" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="四房" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="转生BOSS" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="特殊BOSS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="存档挑战" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="虚空之影" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="修正表" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="解锁条件" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="示例" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="轮换怪血量修正" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3498,6 +3499,76 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>模式</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>难度</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>波次</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>轮换位置</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>最终HP</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>证据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>丰饶</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1420000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>用户确认2026-10-26丰饶N10第8波飞行小怪142万</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Correct rich N10 wave eight flying monster attack to 160 thousand
</commit_message>
<xml_diff>
--- a/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
+++ b/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
@@ -24,7 +24,7 @@
     <sheet name="修正表" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="解锁条件" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="示例" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="轮换怪血量修正" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="轮换怪属性修正" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3505,7 +3505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3536,6 +3536,11 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>最终攻击</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>证据</t>
         </is>
       </c>
@@ -3558,9 +3563,12 @@
       <c r="E2" t="n">
         <v>1420000</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>用户确认2026-10-26丰饶N10第8波飞行小怪142万</t>
+      <c r="F2" t="n">
+        <v>160000</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>用户确认2026-10-26丰饶N10第8波飞行小怪生命142万、攻击16万</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance(rebirth): strengthen rich mode bosses without changing other encounters
</commit_message>
<xml_diff>
--- a/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
+++ b/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
@@ -25,6 +25,7 @@
     <sheet name="解锁条件" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="示例" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="轮换怪属性修正" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="转生模式调优" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3577,6 +3578,75 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>模式</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>生命倍率</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>攻击倍率</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>护甲倍率</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>丰饶</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-28用户要求加强丰饶转生怪；首轮调优在原难度公式后仅对转生BOSS乘一次，幅度为本轮实现选择，待实战确认。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix(rebirth): refresh selected difficulty previews and restore verified v3 stats
</commit_message>
<xml_diff>
--- a/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
+++ b/data/balance/human_spec_v3/接入规格_人话版_v3.xlsx
@@ -25,7 +25,6 @@
     <sheet name="解锁条件" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="示例" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="轮换怪属性修正" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="转生模式调优" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3578,75 +3577,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="100" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>模式</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>生命倍率</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>攻击倍率</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>护甲倍率</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>丰饶</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-28用户要求加强丰饶转生怪；首轮调优在原难度公式后仅对转生BOSS乘一次，幅度为本轮实现选择，待实战确认。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>